<commit_message>
Update Online Practice Excel.xlsx
</commit_message>
<xml_diff>
--- a/Daily Excel/Online Practice Excel.xlsx
+++ b/Daily Excel/Online Practice Excel.xlsx
@@ -5,15 +5,15 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d58d4d655bee1e81/Desktop/Daily Excel/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d58d4d655bee1e81/Desktop/Github/Daily_practice/Daily Excel/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="98" documentId="11_F25DC773A252ABDACC1048BD89DC52D45ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8C65BA7-0FEC-4EED-A016-55B25A984EAD}"/>
+  <xr:revisionPtr revIDLastSave="116" documentId="11_F25DC773A252ABDACC1048BD89DC52D45ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D1AF4BA-4F09-4B88-8B18-6FF301A2FA2C}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Practice" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -61,7 +61,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="429" uniqueCount="352">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="401">
   <si>
     <t>Double-click on cell A1 in the spreadsheet editor. Replace the placeholder text with:</t>
   </si>
@@ -1210,6 +1210,153 @@
   <si>
     <t>3. In G4, calculate the weighted average unit price:</t>
   </si>
+  <si>
+    <t>Use VLOOKUP to find an employee’s department</t>
+  </si>
+  <si>
+    <t>VLOOKUP(lookup_value, table_array, col_index_num, [range_lookup])</t>
+  </si>
+  <si>
+    <t>Directory</t>
+  </si>
+  <si>
+    <t>IT</t>
+  </si>
+  <si>
+    <t>Payroll</t>
+  </si>
+  <si>
+    <t>Lookup</t>
+  </si>
+  <si>
+    <t>Department (fill this)</t>
+  </si>
+  <si>
+    <t>HLOOKUP(lookup_value, table_array, row_index_num, [range_lookup])</t>
+  </si>
+  <si>
+    <t>HLOOKUP for quarterly targets</t>
+  </si>
+  <si>
+    <t>3. Return the sales target from row 2 of the table.</t>
+  </si>
+  <si>
+    <t>Metric</t>
+  </si>
+  <si>
+    <t>Sales target</t>
+  </si>
+  <si>
+    <t>Target</t>
+  </si>
+  <si>
+    <t>1. Click cell B11.</t>
+  </si>
+  <si>
+    <t>2. Type a VLOOKUP formula that uses the employee ID in A11 and searches the directory in A3:B7.</t>
+  </si>
+  <si>
+    <t>3. Return the Department from the directory (the second column of the directory table).</t>
+  </si>
+  <si>
+    <t>4. Use exact match so Excel only matches the exact employee ID.</t>
+  </si>
+  <si>
+    <t>5. Lock the directory range with $ so you can copy the formula.</t>
+  </si>
+  <si>
+    <t>6. Copy your formula down from B11 to B14.</t>
+  </si>
+  <si>
+    <t>1. Click cell B5.</t>
+  </si>
+  <si>
+    <t>2. Write an HLOOKUP formula that looks up the quarter in B4 within the targets table in A1:E2.</t>
+  </si>
+  <si>
+    <t>4. Use FALSE for an exact match.</t>
+  </si>
+  <si>
+    <t>VLOOKUP with approximate match</t>
+  </si>
+  <si>
+    <t>Shipping teams often price delivery in tiers (for example: 0–1 lb, 1–5 lb, 5–10 lb, and so on). In Excel, this is a classic use case for VLOOKUP with an approximate match.</t>
+  </si>
+  <si>
+    <t>Requirements:</t>
+  </si>
+  <si>
+    <t>2. Lock the rate table range so you can copy the formula down.</t>
+  </si>
+  <si>
+    <t>Shipping rate lookup (approximate match)</t>
+  </si>
+  <si>
+    <t>Calculate a per-pound shipping rate based on package weight using VLOOKUP with approximate match (TRUE).</t>
+  </si>
+  <si>
+    <t>Orders</t>
+  </si>
+  <si>
+    <t>Rate table</t>
+  </si>
+  <si>
+    <t>Order #</t>
+  </si>
+  <si>
+    <t>Zone</t>
+  </si>
+  <si>
+    <t>Weight (lb)</t>
+  </si>
+  <si>
+    <t>Rate ($/lb)</t>
+  </si>
+  <si>
+    <t>Shipping cost</t>
+  </si>
+  <si>
+    <t>Min weight (lb)</t>
+  </si>
+  <si>
+    <t>SO-10421</t>
+  </si>
+  <si>
+    <t>Domestic</t>
+  </si>
+  <si>
+    <t>SO-10422</t>
+  </si>
+  <si>
+    <t>SO-10423</t>
+  </si>
+  <si>
+    <t>Canada</t>
+  </si>
+  <si>
+    <t>SO-10424</t>
+  </si>
+  <si>
+    <t>EU</t>
+  </si>
+  <si>
+    <t>SO-10425</t>
+  </si>
+  <si>
+    <t>A list of orders with package weights in C5:C9</t>
+  </si>
+  <si>
+    <t>A tiered rate table in G5:H9 (minimum weight → rate per lb)</t>
+  </si>
+  <si>
+    <t>Fill in D5:D9 with a formula that looks up the correct Rate ($/lb) based on each row’s Weight (lb).</t>
+  </si>
+  <si>
+    <t>1. Use VLOOKUP with approximate match (TRUE) so each weight picks the highest tier that is less than or equal to the weight.</t>
+  </si>
+  <si>
+    <t>3. Copy your formula from D5 down through D9.</t>
+  </si>
 </sst>
 </file>
 
@@ -1218,7 +1365,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="&quot;₹&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1240,8 +1387,15 @@
       <family val="2"/>
       <scheme val="major"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF555555"/>
+      <name val="Calibri Light"/>
+      <family val="2"/>
+      <scheme val="major"/>
+    </font>
   </fonts>
-  <fills count="12">
+  <fills count="13">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1308,6 +1462,12 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF7F7F7"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -1321,7 +1481,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -1390,12 +1550,6 @@
     <xf numFmtId="9" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1422,6 +1576,18 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="12" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1703,7 +1869,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:W322"/>
+  <dimension ref="A1:W385"/>
   <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="149.88671875" style="1" bestFit="1" customWidth="1"/>
@@ -1716,18 +1882,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A1" s="26" t="s">
+      <c r="A1" s="24" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="27"/>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="27"/>
-      <c r="H1" s="27"/>
-      <c r="I1" s="27"/>
-      <c r="J1" s="27"/>
+      <c r="B1" s="25"/>
+      <c r="C1" s="25"/>
+      <c r="D1" s="25"/>
+      <c r="E1" s="25"/>
+      <c r="F1" s="25"/>
+      <c r="G1" s="25"/>
+      <c r="H1" s="25"/>
+      <c r="I1" s="25"/>
+      <c r="J1" s="25"/>
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.3">
       <c r="B3" s="1">
@@ -1736,7 +1902,7 @@
       </c>
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="26" t="s">
         <v>213</v>
       </c>
     </row>
@@ -1792,31 +1958,31 @@
       </c>
     </row>
     <row r="16" spans="1:23" x14ac:dyDescent="0.3">
-      <c r="A16" s="28" t="s">
+      <c r="A16" s="26" t="s">
         <v>28</v>
       </c>
-      <c r="B16" s="29"/>
-      <c r="C16" s="29"/>
-      <c r="D16" s="29"/>
-      <c r="E16" s="29"/>
-      <c r="F16" s="29"/>
-      <c r="G16" s="29"/>
-      <c r="H16" s="29"/>
-      <c r="I16" s="29"/>
-      <c r="J16" s="29"/>
-      <c r="K16" s="29"/>
-      <c r="L16" s="29"/>
-      <c r="M16" s="29"/>
-      <c r="N16" s="29"/>
-      <c r="O16" s="29"/>
-      <c r="P16" s="29"/>
-      <c r="Q16" s="29"/>
-      <c r="R16" s="29"/>
-      <c r="S16" s="29"/>
-      <c r="T16" s="29"/>
-      <c r="U16" s="29"/>
-      <c r="V16" s="29"/>
-      <c r="W16" s="29"/>
+      <c r="B16" s="27"/>
+      <c r="C16" s="27"/>
+      <c r="D16" s="27"/>
+      <c r="E16" s="27"/>
+      <c r="F16" s="27"/>
+      <c r="G16" s="27"/>
+      <c r="H16" s="27"/>
+      <c r="I16" s="27"/>
+      <c r="J16" s="27"/>
+      <c r="K16" s="27"/>
+      <c r="L16" s="27"/>
+      <c r="M16" s="27"/>
+      <c r="N16" s="27"/>
+      <c r="O16" s="27"/>
+      <c r="P16" s="27"/>
+      <c r="Q16" s="27"/>
+      <c r="R16" s="27"/>
+      <c r="S16" s="27"/>
+      <c r="T16" s="27"/>
+      <c r="U16" s="27"/>
+      <c r="V16" s="27"/>
+      <c r="W16" s="27"/>
     </row>
     <row r="18" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A18" s="4">
@@ -1853,31 +2019,31 @@
       </c>
     </row>
     <row r="26" spans="1:23" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A26" s="28" t="s">
+      <c r="A26" s="26" t="s">
         <v>212</v>
       </c>
-      <c r="B26" s="29"/>
-      <c r="C26" s="29"/>
-      <c r="D26" s="29"/>
-      <c r="E26" s="29"/>
-      <c r="F26" s="29"/>
-      <c r="G26" s="29"/>
-      <c r="H26" s="29"/>
-      <c r="I26" s="29"/>
-      <c r="J26" s="29"/>
-      <c r="K26" s="29"/>
-      <c r="L26" s="29"/>
-      <c r="M26" s="29"/>
-      <c r="N26" s="29"/>
-      <c r="O26" s="29"/>
-      <c r="P26" s="29"/>
-      <c r="Q26" s="29"/>
-      <c r="R26" s="29"/>
-      <c r="S26" s="29"/>
-      <c r="T26" s="29"/>
-      <c r="U26" s="29"/>
-      <c r="V26" s="29"/>
-      <c r="W26" s="29"/>
+      <c r="B26" s="27"/>
+      <c r="C26" s="27"/>
+      <c r="D26" s="27"/>
+      <c r="E26" s="27"/>
+      <c r="F26" s="27"/>
+      <c r="G26" s="27"/>
+      <c r="H26" s="27"/>
+      <c r="I26" s="27"/>
+      <c r="J26" s="27"/>
+      <c r="K26" s="27"/>
+      <c r="L26" s="27"/>
+      <c r="M26" s="27"/>
+      <c r="N26" s="27"/>
+      <c r="O26" s="27"/>
+      <c r="P26" s="27"/>
+      <c r="Q26" s="27"/>
+      <c r="R26" s="27"/>
+      <c r="S26" s="27"/>
+      <c r="T26" s="27"/>
+      <c r="U26" s="27"/>
+      <c r="V26" s="27"/>
+      <c r="W26" s="27"/>
     </row>
     <row r="27" spans="1:23" x14ac:dyDescent="0.3">
       <c r="A27" s="7" t="s">
@@ -1990,7 +2156,7 @@
       <c r="D34" s="9"/>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A35" s="28" t="s">
+      <c r="A35" s="26" t="s">
         <v>215</v>
       </c>
     </row>
@@ -2095,7 +2261,7 @@
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A47" s="30" t="s">
+      <c r="A47" s="28" t="s">
         <v>27</v>
       </c>
     </row>
@@ -2298,7 +2464,7 @@
       </c>
     </row>
     <row r="63" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A63" s="30" t="s">
+      <c r="A63" s="28" t="s">
         <v>44</v>
       </c>
     </row>
@@ -2437,7 +2603,7 @@
       </c>
     </row>
     <row r="76" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A76" s="30" t="s">
+      <c r="A76" s="28" t="s">
         <v>71</v>
       </c>
     </row>
@@ -2527,7 +2693,7 @@
       </c>
     </row>
     <row r="89" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A89" s="30" t="s">
+      <c r="A89" s="28" t="s">
         <v>84</v>
       </c>
     </row>
@@ -2627,7 +2793,7 @@
       </c>
     </row>
     <row r="101" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A101" s="30" t="s">
+      <c r="A101" s="28" t="s">
         <v>101</v>
       </c>
     </row>
@@ -2764,7 +2930,7 @@
       </c>
     </row>
     <row r="114" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A114" s="30" t="s">
+      <c r="A114" s="28" t="s">
         <v>111</v>
       </c>
     </row>
@@ -2895,7 +3061,7 @@
       <c r="A127" s="4"/>
     </row>
     <row r="128" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A128" s="31" t="s">
+      <c r="A128" s="29" t="s">
         <v>130</v>
       </c>
     </row>
@@ -3024,7 +3190,7 @@
       <c r="A140" s="4"/>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A141" s="30" t="s">
+      <c r="A141" s="28" t="s">
         <v>139</v>
       </c>
     </row>
@@ -3122,7 +3288,7 @@
       <c r="B151" s="4"/>
     </row>
     <row r="152" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A152" s="31" t="s">
+      <c r="A152" s="29" t="s">
         <v>145</v>
       </c>
       <c r="B152" s="4"/>
@@ -3233,7 +3399,7 @@
       <c r="A162" s="4"/>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A163" s="31" t="s">
+      <c r="A163" s="29" t="s">
         <v>164</v>
       </c>
     </row>
@@ -3260,13 +3426,13 @@
       <c r="A169" s="10" t="s">
         <v>166</v>
       </c>
-      <c r="B169" s="32" t="s">
+      <c r="B169" s="30" t="s">
         <v>198</v>
       </c>
       <c r="C169" s="10" t="s">
         <v>167</v>
       </c>
-      <c r="D169" s="32" t="s">
+      <c r="D169" s="30" t="s">
         <v>199</v>
       </c>
     </row>
@@ -3411,7 +3577,7 @@
       </c>
     </row>
     <row r="181" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A181" s="31" t="s">
+      <c r="A181" s="29" t="s">
         <v>200</v>
       </c>
     </row>
@@ -3492,7 +3658,7 @@
       </c>
     </row>
     <row r="192" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A192" s="31" t="s">
+      <c r="A192" s="29" t="s">
         <v>217</v>
       </c>
     </row>
@@ -3693,7 +3859,7 @@
       <c r="A211" s="2"/>
     </row>
     <row r="212" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A212" s="31" t="s">
+      <c r="A212" s="29" t="s">
         <v>233</v>
       </c>
     </row>
@@ -3839,7 +4005,7 @@
       </c>
     </row>
     <row r="223" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A223" s="31" t="s">
+      <c r="A223" s="29" t="s">
         <v>252</v>
       </c>
     </row>
@@ -3963,16 +4129,16 @@
         <f>_xlfn.XLOOKUP(B235,A227:A233,C227:C233,0)</f>
         <v>Office equipment</v>
       </c>
-      <c r="C236" s="24" t="str">
+      <c r="C236" s="33" t="str">
         <f ca="1">_xlfn.FORMULATEXT(B236)</f>
         <v>=XLOOKUP(B235,A227:A233,C227:C233,0)</v>
       </c>
     </row>
     <row r="237" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="C237" s="24"/>
+      <c r="C237" s="33"/>
     </row>
     <row r="238" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A238" s="31" t="s">
+      <c r="A238" s="29" t="s">
         <v>274</v>
       </c>
     </row>
@@ -4134,14 +4300,14 @@
       </c>
     </row>
     <row r="256" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="B256" s="25" t="str">
+      <c r="B256" s="34" t="str">
         <f ca="1">_xlfn.FORMULATEXT(C251)</f>
         <v>=XLOOKUP(A251,A$242:A$248,$C$242:$C$248,0)</v>
       </c>
-      <c r="C256" s="25"/>
+      <c r="C256" s="34"/>
     </row>
     <row r="258" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A258" s="31" t="s">
+      <c r="A258" s="29" t="s">
         <v>292</v>
       </c>
     </row>
@@ -4281,7 +4447,7 @@
       </c>
     </row>
     <row r="270" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A270" s="31" t="s">
+      <c r="A270" s="29" t="s">
         <v>303</v>
       </c>
     </row>
@@ -4415,7 +4581,7 @@
       </c>
     </row>
     <row r="283" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A283" s="31" t="s">
+      <c r="A283" s="29" t="s">
         <v>308</v>
       </c>
       <c r="D283" s="1" t="str">
@@ -4564,7 +4730,7 @@
       </c>
     </row>
     <row r="301" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A301" s="31" t="s">
+      <c r="A301" s="29" t="s">
         <v>326</v>
       </c>
     </row>
@@ -4574,15 +4740,15 @@
       </c>
     </row>
     <row r="303" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A303" s="33"/>
+      <c r="A303" s="31"/>
     </row>
     <row r="304" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A304" s="33" t="s">
+      <c r="A304" s="31" t="s">
         <v>347</v>
       </c>
     </row>
     <row r="305" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A305" s="33" t="s">
+      <c r="A305" s="31" t="s">
         <v>348</v>
       </c>
     </row>
@@ -4595,25 +4761,25 @@
       </c>
     </row>
     <row r="308" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A308" s="33"/>
+      <c r="A308" s="31"/>
     </row>
     <row r="309" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A309" s="33" t="s">
+      <c r="A309" s="31" t="s">
         <v>349</v>
       </c>
     </row>
     <row r="310" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A310" s="33" t="s">
+      <c r="A310" s="31" t="s">
         <v>350</v>
       </c>
     </row>
     <row r="311" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A311" s="33" t="s">
+      <c r="A311" s="31" t="s">
         <v>351</v>
       </c>
     </row>
     <row r="312" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A312" s="34" t="s">
+      <c r="A312" s="32" t="s">
         <v>328</v>
       </c>
     </row>
@@ -4787,10 +4953,506 @@
       <c r="F322" s="4"/>
       <c r="G322" s="4"/>
     </row>
+    <row r="324" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A324" s="29" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="325" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A325" s="16" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="326" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A326" s="31" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="327" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A327" s="31" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="328" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A328" s="31" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="329" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A329" s="31" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="330" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A330" s="31" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="331" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A331" s="31" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="333" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A333" s="4" t="s">
+        <v>354</v>
+      </c>
+      <c r="B333" s="4"/>
+    </row>
+    <row r="334" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A334" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B334" s="7" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="335" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A335" s="4">
+        <v>1040</v>
+      </c>
+      <c r="B335" s="4" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="336" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A336" s="4">
+        <v>1042</v>
+      </c>
+      <c r="B336" s="4" t="s">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="337" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A337" s="4">
+        <v>1051</v>
+      </c>
+      <c r="B337" s="4" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="338" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A338" s="4">
+        <v>1063</v>
+      </c>
+      <c r="B338" s="4" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="339" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A339" s="4">
+        <v>1038</v>
+      </c>
+      <c r="B339" s="4" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="340" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A340" s="4"/>
+      <c r="B340" s="4"/>
+    </row>
+    <row r="341" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A341" s="4" t="s">
+        <v>357</v>
+      </c>
+      <c r="B341" s="4"/>
+    </row>
+    <row r="342" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A342" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B342" s="7" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="343" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A343" s="4">
+        <v>1042</v>
+      </c>
+      <c r="B343" s="5" t="str">
+        <f>VLOOKUP(A343,$A$335:$B$339,2,0)</f>
+        <v>HR</v>
+      </c>
+      <c r="C343" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(B343)</f>
+        <v>=VLOOKUP(A343,$A$335:$B$339,2,0)</v>
+      </c>
+    </row>
+    <row r="344" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A344" s="4">
+        <v>1038</v>
+      </c>
+      <c r="B344" s="5" t="str">
+        <f t="shared" ref="B344:B346" si="16">VLOOKUP(A344,$A$335:$B$339,2,0)</f>
+        <v>Payroll</v>
+      </c>
+    </row>
+    <row r="345" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A345" s="4">
+        <v>1051</v>
+      </c>
+      <c r="B345" s="5" t="str">
+        <f t="shared" si="16"/>
+        <v>IT</v>
+      </c>
+    </row>
+    <row r="346" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A346" s="4">
+        <v>1040</v>
+      </c>
+      <c r="B346" s="5" t="str">
+        <f t="shared" si="16"/>
+        <v>Finance</v>
+      </c>
+    </row>
+    <row r="347" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A347" s="4"/>
+    </row>
+    <row r="348" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A348" s="29" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="349" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A349" s="16" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="350" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A350" s="31" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="351" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A351" s="31" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="352" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A352" s="31" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="353" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A353" s="31" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="355" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A355" s="7" t="s">
+        <v>362</v>
+      </c>
+      <c r="B355" s="7" t="s">
+        <v>314</v>
+      </c>
+      <c r="C355" s="7" t="s">
+        <v>315</v>
+      </c>
+      <c r="D355" s="7" t="s">
+        <v>316</v>
+      </c>
+      <c r="E355" s="7" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="356" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A356" s="4" t="s">
+        <v>363</v>
+      </c>
+      <c r="B356" s="4">
+        <v>85000</v>
+      </c>
+      <c r="C356" s="4">
+        <v>95000</v>
+      </c>
+      <c r="D356" s="4">
+        <v>110000</v>
+      </c>
+      <c r="E356" s="4">
+        <v>120000</v>
+      </c>
+    </row>
+    <row r="357" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C357" s="4"/>
+      <c r="D357" s="4"/>
+      <c r="E357" s="4"/>
+    </row>
+    <row r="358" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A358" s="1" t="s">
+        <v>310</v>
+      </c>
+      <c r="B358" s="1" t="s">
+        <v>316</v>
+      </c>
+      <c r="C358" s="5">
+        <f>HLOOKUP(B358,A355:E356,2,0)</f>
+        <v>110000</v>
+      </c>
+      <c r="D358" s="4"/>
+      <c r="E358" s="4"/>
+    </row>
+    <row r="359" spans="1:5" ht="26.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A359" s="1" t="s">
+        <v>364</v>
+      </c>
+      <c r="C359" s="33" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(C358)</f>
+        <v>=HLOOKUP(B358,A355:E356,2,0)</v>
+      </c>
+      <c r="D359" s="4"/>
+      <c r="E359" s="4"/>
+    </row>
+    <row r="360" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C360" s="33"/>
+    </row>
+    <row r="362" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A362" s="29" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="363" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A363" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="364" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A364" s="31" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="365" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A365" s="31" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="367" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A367" s="4" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="368" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A368" s="16"/>
+    </row>
+    <row r="369" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A369" s="4" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="370" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A370" s="31"/>
+    </row>
+    <row r="371" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A371" s="31" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="372" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A372" s="31" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="373" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A373" s="31" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="375" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A375" s="4" t="s">
+        <v>378</v>
+      </c>
+      <c r="B375" s="4"/>
+      <c r="C375" s="4"/>
+      <c r="D375" s="4"/>
+      <c r="E375" s="4"/>
+      <c r="F375" s="4"/>
+      <c r="G375" s="4"/>
+      <c r="H375" s="4"/>
+    </row>
+    <row r="376" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A376" s="35" t="s">
+        <v>379</v>
+      </c>
+      <c r="B376" s="4"/>
+      <c r="C376" s="4"/>
+      <c r="D376" s="4"/>
+      <c r="E376" s="4"/>
+      <c r="F376" s="4"/>
+      <c r="G376" s="4"/>
+      <c r="H376" s="4"/>
+    </row>
+    <row r="377" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A377" s="36" t="s">
+        <v>380</v>
+      </c>
+      <c r="B377" s="4"/>
+      <c r="C377" s="4"/>
+      <c r="E377" s="4"/>
+      <c r="F377" s="4"/>
+      <c r="G377" s="36" t="s">
+        <v>381</v>
+      </c>
+      <c r="H377" s="4"/>
+    </row>
+    <row r="378" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A378" s="7" t="s">
+        <v>382</v>
+      </c>
+      <c r="B378" s="7" t="s">
+        <v>383</v>
+      </c>
+      <c r="C378" s="7" t="s">
+        <v>384</v>
+      </c>
+      <c r="D378" s="7" t="s">
+        <v>385</v>
+      </c>
+      <c r="E378" s="7" t="s">
+        <v>386</v>
+      </c>
+      <c r="F378" s="4"/>
+      <c r="G378" s="7" t="s">
+        <v>387</v>
+      </c>
+      <c r="H378" s="7" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="379" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A379" s="4" t="s">
+        <v>388</v>
+      </c>
+      <c r="B379" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="C379" s="4">
+        <v>0.8</v>
+      </c>
+      <c r="D379" s="5">
+        <f>VLOOKUP(C379,G379:H383,2,1)</f>
+        <v>6.5</v>
+      </c>
+      <c r="E379" s="4">
+        <v>5.2</v>
+      </c>
+      <c r="F379" s="4"/>
+      <c r="G379" s="4">
+        <v>0</v>
+      </c>
+      <c r="H379" s="4">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="380" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A380" s="4" t="s">
+        <v>390</v>
+      </c>
+      <c r="B380" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="C380" s="4">
+        <v>2.4</v>
+      </c>
+      <c r="D380" s="5">
+        <f t="shared" ref="D380:D383" si="17">VLOOKUP(C380,G380:H384,2,1)</f>
+        <v>5.75</v>
+      </c>
+      <c r="E380" s="4">
+        <v>13.8</v>
+      </c>
+      <c r="F380" s="4"/>
+      <c r="G380" s="4">
+        <v>1</v>
+      </c>
+      <c r="H380" s="4">
+        <v>5.75</v>
+      </c>
+    </row>
+    <row r="381" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A381" s="4" t="s">
+        <v>391</v>
+      </c>
+      <c r="B381" s="4" t="s">
+        <v>392</v>
+      </c>
+      <c r="C381" s="4">
+        <v>6.2</v>
+      </c>
+      <c r="D381" s="5">
+        <f>VLOOKUP(C381,G381:H385,2,1)</f>
+        <v>5</v>
+      </c>
+      <c r="E381" s="4">
+        <v>31</v>
+      </c>
+      <c r="F381" s="4"/>
+      <c r="G381" s="4">
+        <v>5</v>
+      </c>
+      <c r="H381" s="4">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="382" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A382" s="4" t="s">
+        <v>393</v>
+      </c>
+      <c r="B382" s="4" t="s">
+        <v>394</v>
+      </c>
+      <c r="C382" s="4">
+        <v>12</v>
+      </c>
+      <c r="D382" s="5">
+        <f t="shared" si="17"/>
+        <v>4.25</v>
+      </c>
+      <c r="E382" s="4">
+        <v>51</v>
+      </c>
+      <c r="F382" s="4"/>
+      <c r="G382" s="4">
+        <v>10</v>
+      </c>
+      <c r="H382" s="4">
+        <v>4.25</v>
+      </c>
+    </row>
+    <row r="383" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A383" s="4" t="s">
+        <v>395</v>
+      </c>
+      <c r="B383" s="4" t="s">
+        <v>389</v>
+      </c>
+      <c r="C383" s="4">
+        <v>24.5</v>
+      </c>
+      <c r="D383" s="5">
+        <f t="shared" si="17"/>
+        <v>3.75</v>
+      </c>
+      <c r="E383" s="4">
+        <v>91.875</v>
+      </c>
+      <c r="F383" s="4"/>
+      <c r="G383" s="4">
+        <v>20</v>
+      </c>
+      <c r="H383" s="4">
+        <v>3.75</v>
+      </c>
+    </row>
+    <row r="385" spans="4:4" x14ac:dyDescent="0.3">
+      <c r="D385" s="1" t="str">
+        <f ca="1">_xlfn.FORMULATEXT(D379)</f>
+        <v>=VLOOKUP(C379,G379:H383,2,1)</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="C236:C237"/>
     <mergeCell ref="B256:C256"/>
+    <mergeCell ref="C359:C360"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>